<commit_message>
Crear una control de proyecto en formato Excel
</commit_message>
<xml_diff>
--- a/Proyecto_Diaring.xlsx
+++ b/Proyecto_Diaring.xlsx
@@ -9,10 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9735"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9735" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="¿Quiénes somos" sheetId="1" r:id="rId1"/>
+    <sheet name="Tutoriales" sheetId="2" r:id="rId2"/>
+    <sheet name="Paleta de colores" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Misión</t>
   </si>
@@ -45,6 +47,18 @@
   </si>
   <si>
     <t>Hacer carrusel con las fotos del colegio</t>
+  </si>
+  <si>
+    <t>Actividades:</t>
+  </si>
+  <si>
+    <t>FALTA DEFINIR</t>
+  </si>
+  <si>
+    <t>¿Qué son Tutoriales?</t>
+  </si>
+  <si>
+    <t>Es un apartado de el sitio web Diaring en el cual los usuarios pueden explorar a profundidad las funcionalidades de el sitio web y los conceptos claves que lo componen a traves de links a sitios externos</t>
   </si>
 </sst>
 </file>
@@ -88,9 +102,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -190,6 +207,55 @@
         <a:xfrm>
           <a:off x="762000" y="4000501"/>
           <a:ext cx="2507753" cy="1028700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>5336232</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="762000" y="190500"/>
+          <a:ext cx="5336232" cy="2247900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -510,4 +576,48 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B15:B21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="112.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="B17" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>